<commit_message>
Show Tunis Landing values
</commit_message>
<xml_diff>
--- a/templates/Tunis_OPEX_2027.xlsx
+++ b/templates/Tunis_OPEX_2027.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tunis OPEX 2027" sheetId="2" r:id="Re54122d4af8f4af3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tunis OPEX 2027" sheetId="2" r:id="R988e6bdba4e74b57"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1638,19 +1638,19 @@
       <x:c r="C2" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D2" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E2" s="4" t="n">
-        <x:v>0</x:v>
+      <x:c r="D2" s="4">
+        <x:v>25651.324717200001</x:v>
+      </x:c>
+      <x:c r="E2" s="4">
+        <x:v>14314.6255</x:v>
       </x:c>
       <x:c r="F2" s="4" t="n">
         <x:f>E2/7*5</x:f>
-        <x:v>0</x:v>
+        <x:v>10224.7325</x:v>
       </x:c>
       <x:c r="G2" s="4" t="n">
         <x:f>F2+E2</x:f>
-        <x:v>0</x:v>
+        <x:v>24539.358</x:v>
       </x:c>
       <x:c r="H2" s="2">
         <x:v>0</x:v>
@@ -1703,10 +1703,10 @@
       <x:c r="C3" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D3" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E3" s="4" t="n">
+      <x:c r="D3" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E3" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F3" s="4">
@@ -1766,10 +1766,10 @@
       <x:c r="C4" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D4" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E4" s="4" t="n">
+      <x:c r="D4" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E4" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F4" s="4">
@@ -1829,10 +1829,10 @@
       <x:c r="C5" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D5" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E5" s="4" t="n">
+      <x:c r="D5" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E5" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F5" s="4">
@@ -1892,10 +1892,10 @@
       <x:c r="C6" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D6" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E6" s="4" t="n">
+      <x:c r="D6" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E6" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F6" s="4">
@@ -1955,10 +1955,10 @@
       <x:c r="C7" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D7" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E7" s="4" t="n">
+      <x:c r="D7" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E7" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F7" s="4">
@@ -2018,10 +2018,10 @@
       <x:c r="C8" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D8" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E8" s="4" t="n">
+      <x:c r="D8" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E8" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F8" s="4">
@@ -2081,10 +2081,10 @@
       <x:c r="C9" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D9" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E9" s="4" t="n">
+      <x:c r="D9" s="4">
+        <x:v>98.28</x:v>
+      </x:c>
+      <x:c r="E9" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F9" s="4">
@@ -2144,10 +2144,10 @@
       <x:c r="C10" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D10" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E10" s="4" t="n">
+      <x:c r="D10" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E10" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F10" s="4">
@@ -2207,10 +2207,10 @@
       <x:c r="C11" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D11" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E11" s="4" t="n">
+      <x:c r="D11" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E11" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F11" s="4">
@@ -2270,10 +2270,10 @@
       <x:c r="C12" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D12" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E12" s="4" t="n">
+      <x:c r="D12" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E12" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F12" s="4">
@@ -2333,10 +2333,10 @@
       <x:c r="C13" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D13" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E13" s="4" t="n">
+      <x:c r="D13" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E13" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F13" s="4">
@@ -2396,10 +2396,10 @@
       <x:c r="C14" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D14" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E14" s="4" t="n">
+      <x:c r="D14" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E14" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F14" s="4">
@@ -2459,10 +2459,10 @@
       <x:c r="C15" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D15" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E15" s="4" t="n">
+      <x:c r="D15" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E15" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F15" s="4">
@@ -2522,10 +2522,10 @@
       <x:c r="C16" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D16" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E16" s="4" t="n">
+      <x:c r="D16" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E16" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F16" s="4">
@@ -2585,10 +2585,10 @@
       <x:c r="C17" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D17" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E17" s="4" t="n">
+      <x:c r="D17" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E17" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F17" s="4">
@@ -2648,10 +2648,10 @@
       <x:c r="C18" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D18" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E18" s="4" t="n">
+      <x:c r="D18" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E18" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F18" s="4">
@@ -2711,10 +2711,10 @@
       <x:c r="C19" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D19" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E19" s="4" t="n">
+      <x:c r="D19" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E19" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F19" s="4">
@@ -2774,10 +2774,10 @@
       <x:c r="C20" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D20" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E20" s="4" t="n">
+      <x:c r="D20" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E20" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F20" s="4">
@@ -2837,10 +2837,10 @@
       <x:c r="C21" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D21" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E21" s="4" t="n">
+      <x:c r="D21" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E21" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F21" s="4">
@@ -2900,10 +2900,10 @@
       <x:c r="C22" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D22" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E22" s="4" t="n">
+      <x:c r="D22" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E22" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F22" s="4">
@@ -2963,10 +2963,10 @@
       <x:c r="C23" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D23" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E23" s="4" t="n">
+      <x:c r="D23" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E23" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F23" s="4">
@@ -3026,10 +3026,10 @@
       <x:c r="C24" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D24" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E24" s="4" t="n">
+      <x:c r="D24" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E24" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F24" s="4">
@@ -3089,10 +3089,10 @@
       <x:c r="C25" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D25" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E25" s="4" t="n">
+      <x:c r="D25" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E25" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F25" s="4">
@@ -3152,10 +3152,10 @@
       <x:c r="C26" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D26" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E26" s="4" t="n">
+      <x:c r="D26" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E26" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F26" s="4">
@@ -3215,10 +3215,10 @@
       <x:c r="C27" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D27" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E27" s="4" t="n">
+      <x:c r="D27" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E27" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F27" s="4">
@@ -3278,10 +3278,10 @@
       <x:c r="C28" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D28" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E28" s="4" t="n">
+      <x:c r="D28" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E28" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F28" s="4">
@@ -3341,10 +3341,10 @@
       <x:c r="C29" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D29" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E29" s="4" t="n">
+      <x:c r="D29" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E29" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F29" s="4">
@@ -3404,10 +3404,10 @@
       <x:c r="C30" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D30" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E30" s="4" t="n">
+      <x:c r="D30" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E30" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F30" s="4">
@@ -3467,10 +3467,10 @@
       <x:c r="C31" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D31" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E31" s="4" t="n">
+      <x:c r="D31" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E31" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F31" s="4">
@@ -3530,10 +3530,10 @@
       <x:c r="C32" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D32" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E32" s="4" t="n">
+      <x:c r="D32" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E32" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F32" s="4">
@@ -3593,10 +3593,10 @@
       <x:c r="C33" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D33" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E33" s="4" t="n">
+      <x:c r="D33" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E33" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F33" s="4">
@@ -3656,10 +3656,10 @@
       <x:c r="C34" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D34" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E34" s="4" t="n">
+      <x:c r="D34" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E34" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F34" s="4">
@@ -3719,10 +3719,10 @@
       <x:c r="C35" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D35" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E35" s="4" t="n">
+      <x:c r="D35" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E35" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F35" s="4">
@@ -3782,10 +3782,10 @@
       <x:c r="C36" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D36" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E36" s="4" t="n">
+      <x:c r="D36" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E36" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F36" s="4">
@@ -3845,10 +3845,10 @@
       <x:c r="C37" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D37" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E37" s="4" t="n">
+      <x:c r="D37" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E37" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F37" s="4">
@@ -3908,10 +3908,10 @@
       <x:c r="C38" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D38" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E38" s="4" t="n">
+      <x:c r="D38" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E38" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F38" s="4">
@@ -3971,10 +3971,10 @@
       <x:c r="C39" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D39" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E39" s="4" t="n">
+      <x:c r="D39" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E39" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F39" s="4">
@@ -4034,10 +4034,10 @@
       <x:c r="C40" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D40" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E40" s="4" t="n">
+      <x:c r="D40" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E40" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F40" s="4">
@@ -4097,10 +4097,10 @@
       <x:c r="C41" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D41" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E41" s="4" t="n">
+      <x:c r="D41" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E41" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F41" s="4">
@@ -4160,10 +4160,10 @@
       <x:c r="C42" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D42" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E42" s="4" t="n">
+      <x:c r="D42" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E42" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F42" s="4">
@@ -4223,10 +4223,10 @@
       <x:c r="C43" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D43" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E43" s="4" t="n">
+      <x:c r="D43" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E43" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F43" s="4">
@@ -4286,10 +4286,10 @@
       <x:c r="C44" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D44" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E44" s="4" t="n">
+      <x:c r="D44" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E44" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F44" s="4">
@@ -4349,10 +4349,10 @@
       <x:c r="C45" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D45" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E45" s="4" t="n">
+      <x:c r="D45" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E45" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F45" s="4">
@@ -4412,10 +4412,10 @@
       <x:c r="C46" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D46" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E46" s="4" t="n">
+      <x:c r="D46" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E46" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F46" s="4">
@@ -4475,10 +4475,10 @@
       <x:c r="C47" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D47" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E47" s="4" t="n">
+      <x:c r="D47" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E47" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F47" s="4">
@@ -4538,10 +4538,10 @@
       <x:c r="C48" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D48" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E48" s="4" t="n">
+      <x:c r="D48" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E48" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F48" s="4">
@@ -4601,10 +4601,10 @@
       <x:c r="C49" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D49" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E49" s="4" t="n">
+      <x:c r="D49" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E49" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F49" s="4">
@@ -4664,10 +4664,10 @@
       <x:c r="C50" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D50" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E50" s="4" t="n">
+      <x:c r="D50" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E50" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F50" s="4">
@@ -4727,10 +4727,10 @@
       <x:c r="C51" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D51" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E51" s="4" t="n">
+      <x:c r="D51" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E51" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F51" s="4">
@@ -4790,10 +4790,10 @@
       <x:c r="C52" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D52" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E52" s="4" t="n">
+      <x:c r="D52" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E52" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F52" s="4">
@@ -4853,10 +4853,10 @@
       <x:c r="C53" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D53" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E53" s="4" t="n">
+      <x:c r="D53" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E53" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F53" s="4">
@@ -4916,10 +4916,10 @@
       <x:c r="C54" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D54" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E54" s="4" t="n">
+      <x:c r="D54" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E54" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F54" s="4">
@@ -4979,10 +4979,10 @@
       <x:c r="C55" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D55" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E55" s="4" t="n">
+      <x:c r="D55" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E55" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F55" s="4">
@@ -5042,10 +5042,10 @@
       <x:c r="C56" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D56" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E56" s="4" t="n">
+      <x:c r="D56" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E56" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F56" s="4">
@@ -5105,10 +5105,10 @@
       <x:c r="C57" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D57" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E57" s="4" t="n">
+      <x:c r="D57" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E57" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F57" s="4">
@@ -5168,10 +5168,10 @@
       <x:c r="C58" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D58" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E58" s="4" t="n">
+      <x:c r="D58" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E58" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F58" s="4">
@@ -5231,10 +5231,10 @@
       <x:c r="C59" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D59" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E59" s="4" t="n">
+      <x:c r="D59" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E59" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F59" s="4">
@@ -5294,10 +5294,10 @@
       <x:c r="C60" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D60" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E60" s="4" t="n">
+      <x:c r="D60" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E60" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F60" s="4">
@@ -5357,10 +5357,10 @@
       <x:c r="C61" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D61" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E61" s="4" t="n">
+      <x:c r="D61" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E61" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F61" s="4">
@@ -5420,10 +5420,10 @@
       <x:c r="C62" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D62" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E62" s="4" t="n">
+      <x:c r="D62" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E62" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F62" s="4">
@@ -5483,10 +5483,10 @@
       <x:c r="C63" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D63" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E63" s="4" t="n">
+      <x:c r="D63" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E63" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F63" s="4">
@@ -5546,10 +5546,10 @@
       <x:c r="C64" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D64" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E64" s="4" t="n">
+      <x:c r="D64" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E64" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F64" s="4">
@@ -5609,10 +5609,10 @@
       <x:c r="C65" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D65" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E65" s="4" t="n">
+      <x:c r="D65" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E65" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F65" s="4">
@@ -5672,10 +5672,10 @@
       <x:c r="C66" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D66" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E66" s="4" t="n">
+      <x:c r="D66" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E66" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F66" s="4">
@@ -5735,10 +5735,10 @@
       <x:c r="C67" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D67" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E67" s="4" t="n">
+      <x:c r="D67" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E67" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F67" s="4">
@@ -5798,10 +5798,10 @@
       <x:c r="C68" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D68" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E68" s="4" t="n">
+      <x:c r="D68" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E68" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F68" s="4">
@@ -5861,10 +5861,10 @@
       <x:c r="C69" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D69" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E69" s="4" t="n">
+      <x:c r="D69" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E69" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F69" s="4">
@@ -5924,10 +5924,10 @@
       <x:c r="C70" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D70" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E70" s="4" t="n">
+      <x:c r="D70" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E70" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F70" s="4">
@@ -5987,10 +5987,10 @@
       <x:c r="C71" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D71" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E71" s="4" t="n">
+      <x:c r="D71" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E71" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F71" s="4">
@@ -6050,10 +6050,10 @@
       <x:c r="C72" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D72" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E72" s="4" t="n">
+      <x:c r="D72" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E72" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F72" s="4">
@@ -6113,10 +6113,10 @@
       <x:c r="C73" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D73" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E73" s="4" t="n">
+      <x:c r="D73" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E73" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F73" s="4">
@@ -6176,10 +6176,10 @@
       <x:c r="C74" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D74" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E74" s="4" t="n">
+      <x:c r="D74" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E74" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F74" s="4">
@@ -6239,10 +6239,10 @@
       <x:c r="C75" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D75" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E75" s="4" t="n">
+      <x:c r="D75" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E75" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F75" s="4">
@@ -6302,10 +6302,10 @@
       <x:c r="C76" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D76" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E76" s="4" t="n">
+      <x:c r="D76" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E76" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F76" s="4">
@@ -6365,10 +6365,10 @@
       <x:c r="C77" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D77" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E77" s="4" t="n">
+      <x:c r="D77" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E77" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F77" s="4">
@@ -6428,10 +6428,10 @@
       <x:c r="C78" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D78" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E78" s="4" t="n">
+      <x:c r="D78" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E78" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F78" s="4">
@@ -6491,10 +6491,10 @@
       <x:c r="C79" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D79" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E79" s="4" t="n">
+      <x:c r="D79" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E79" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F79" s="4">
@@ -6554,10 +6554,10 @@
       <x:c r="C80" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D80" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E80" s="4" t="n">
+      <x:c r="D80" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E80" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F80" s="4">
@@ -6617,10 +6617,10 @@
       <x:c r="C81" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D81" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E81" s="4" t="n">
+      <x:c r="D81" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E81" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F81" s="4">
@@ -6680,10 +6680,10 @@
       <x:c r="C82" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D82" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E82" s="4" t="n">
+      <x:c r="D82" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E82" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F82" s="4">
@@ -6743,10 +6743,10 @@
       <x:c r="C83" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D83" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E83" s="4" t="n">
+      <x:c r="D83" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E83" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F83" s="4">
@@ -6806,10 +6806,10 @@
       <x:c r="C84" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D84" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E84" s="4" t="n">
+      <x:c r="D84" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E84" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F84" s="4">
@@ -6869,10 +6869,10 @@
       <x:c r="C85" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D85" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E85" s="4" t="n">
+      <x:c r="D85" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E85" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F85" s="4">
@@ -6932,10 +6932,10 @@
       <x:c r="C86" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D86" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E86" s="4" t="n">
+      <x:c r="D86" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E86" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F86" s="4">
@@ -6995,10 +6995,10 @@
       <x:c r="C87" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D87" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E87" s="4" t="n">
+      <x:c r="D87" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E87" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F87" s="4">
@@ -7058,10 +7058,10 @@
       <x:c r="C88" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D88" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E88" s="4" t="n">
+      <x:c r="D88" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E88" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F88" s="4">
@@ -7121,10 +7121,10 @@
       <x:c r="C89" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D89" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E89" s="4" t="n">
+      <x:c r="D89" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E89" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F89" s="4">
@@ -7184,10 +7184,10 @@
       <x:c r="C90" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D90" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E90" s="4" t="n">
+      <x:c r="D90" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E90" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F90" s="4">
@@ -7247,10 +7247,10 @@
       <x:c r="C91" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D91" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E91" s="4" t="n">
+      <x:c r="D91" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E91" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F91" s="4">
@@ -7310,10 +7310,10 @@
       <x:c r="C92" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D92" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E92" s="4" t="n">
+      <x:c r="D92" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E92" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F92" s="4">
@@ -7373,10 +7373,10 @@
       <x:c r="C93" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D93" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E93" s="4" t="n">
+      <x:c r="D93" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E93" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F93" s="4">
@@ -7436,10 +7436,10 @@
       <x:c r="C94" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D94" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E94" s="4" t="n">
+      <x:c r="D94" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E94" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F94" s="4">
@@ -7499,10 +7499,10 @@
       <x:c r="C95" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D95" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E95" s="4" t="n">
+      <x:c r="D95" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E95" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F95" s="4">
@@ -7562,10 +7562,10 @@
       <x:c r="C96" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D96" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E96" s="4" t="n">
+      <x:c r="D96" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E96" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F96" s="4">
@@ -7625,10 +7625,10 @@
       <x:c r="C97" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D97" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E97" s="4" t="n">
+      <x:c r="D97" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E97" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F97" s="4">
@@ -7688,10 +7688,10 @@
       <x:c r="C98" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D98" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E98" s="4" t="n">
+      <x:c r="D98" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E98" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F98" s="4">
@@ -7751,10 +7751,10 @@
       <x:c r="C99" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D99" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E99" s="4" t="n">
+      <x:c r="D99" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E99" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F99" s="4">
@@ -7814,10 +7814,10 @@
       <x:c r="C100" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D100" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E100" s="4" t="n">
+      <x:c r="D100" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E100" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F100" s="4">
@@ -7877,10 +7877,10 @@
       <x:c r="C101" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D101" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E101" s="4" t="n">
+      <x:c r="D101" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E101" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F101" s="4">
@@ -7940,10 +7940,10 @@
       <x:c r="C102" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D102" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E102" s="4" t="n">
+      <x:c r="D102" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E102" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F102" s="4">
@@ -8003,10 +8003,10 @@
       <x:c r="C103" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D103" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E103" s="4" t="n">
+      <x:c r="D103" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E103" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F103" s="4">
@@ -8066,10 +8066,10 @@
       <x:c r="C104" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D104" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E104" s="4" t="n">
+      <x:c r="D104" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E104" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F104" s="4">
@@ -8129,10 +8129,10 @@
       <x:c r="C105" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D105" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E105" s="4" t="n">
+      <x:c r="D105" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E105" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F105" s="4">
@@ -8192,10 +8192,10 @@
       <x:c r="C106" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D106" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E106" s="4" t="n">
+      <x:c r="D106" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E106" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F106" s="4">
@@ -8255,19 +8255,19 @@
       <x:c r="C107" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D107" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E107" s="4" t="n">
-        <x:v>0</x:v>
+      <x:c r="D107" s="4">
+        <x:v>3865.8438000000001</x:v>
+      </x:c>
+      <x:c r="E107" s="4">
+        <x:v>851.54881999999998</x:v>
       </x:c>
       <x:c r="F107" s="4" t="n">
         <x:f>E107/7*5</x:f>
-        <x:v>0</x:v>
+        <x:v>608.2491571428571</x:v>
       </x:c>
       <x:c r="G107" s="4" t="n">
         <x:f>F107+E107</x:f>
-        <x:v>0</x:v>
+        <x:v>1459.7979771428572</x:v>
       </x:c>
       <x:c r="H107" s="2">
         <x:v>0</x:v>
@@ -8320,10 +8320,10 @@
       <x:c r="C108" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D108" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E108" s="4" t="n">
+      <x:c r="D108" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E108" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F108" s="4">
@@ -8383,10 +8383,10 @@
       <x:c r="C109" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D109" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E109" s="4" t="n">
+      <x:c r="D109" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E109" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F109" s="4">
@@ -8446,10 +8446,10 @@
       <x:c r="C110" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D110" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E110" s="4" t="n">
+      <x:c r="D110" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E110" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F110" s="4">
@@ -8509,10 +8509,10 @@
       <x:c r="C111" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D111" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E111" s="4" t="n">
+      <x:c r="D111" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E111" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F111" s="4">
@@ -8572,10 +8572,10 @@
       <x:c r="C112" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D112" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E112" s="4" t="n">
+      <x:c r="D112" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E112" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F112" s="4">
@@ -8635,10 +8635,10 @@
       <x:c r="C113" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D113" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E113" s="4" t="n">
+      <x:c r="D113" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E113" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F113" s="4">
@@ -8698,10 +8698,10 @@
       <x:c r="C114" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D114" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E114" s="4" t="n">
+      <x:c r="D114" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E114" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F114" s="4">
@@ -8761,10 +8761,10 @@
       <x:c r="C115" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D115" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E115" s="4" t="n">
+      <x:c r="D115" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E115" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F115" s="4">
@@ -8824,10 +8824,10 @@
       <x:c r="C116" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D116" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E116" s="4" t="n">
+      <x:c r="D116" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E116" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F116" s="4">
@@ -8887,10 +8887,10 @@
       <x:c r="C117" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D117" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E117" s="4" t="n">
+      <x:c r="D117" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E117" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F117" s="4">
@@ -8950,10 +8950,10 @@
       <x:c r="C118" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D118" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E118" s="4" t="n">
+      <x:c r="D118" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E118" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F118" s="4">
@@ -9013,10 +9013,10 @@
       <x:c r="C119" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D119" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E119" s="4" t="n">
+      <x:c r="D119" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E119" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F119" s="4">
@@ -9076,10 +9076,10 @@
       <x:c r="C120" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D120" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E120" s="4" t="n">
+      <x:c r="D120" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E120" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F120" s="4">
@@ -9139,10 +9139,10 @@
       <x:c r="C121" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D121" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E121" s="4" t="n">
+      <x:c r="D121" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E121" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F121" s="4">
@@ -9202,10 +9202,10 @@
       <x:c r="C122" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D122" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E122" s="4" t="n">
+      <x:c r="D122" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E122" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F122" s="4">
@@ -9265,10 +9265,10 @@
       <x:c r="C123" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D123" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E123" s="4" t="n">
+      <x:c r="D123" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E123" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F123" s="4">
@@ -9328,10 +9328,10 @@
       <x:c r="C124" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D124" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E124" s="4" t="n">
+      <x:c r="D124" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E124" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F124" s="4">
@@ -9391,10 +9391,10 @@
       <x:c r="C125" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D125" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E125" s="4" t="n">
+      <x:c r="D125" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E125" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F125" s="4">
@@ -9454,10 +9454,10 @@
       <x:c r="C126" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D126" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E126" s="4" t="n">
+      <x:c r="D126" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E126" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F126" s="4">
@@ -9517,10 +9517,10 @@
       <x:c r="C127" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D127" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E127" s="4" t="n">
+      <x:c r="D127" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E127" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F127" s="4">
@@ -9580,10 +9580,10 @@
       <x:c r="C128" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D128" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E128" s="4" t="n">
+      <x:c r="D128" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E128" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F128" s="4">
@@ -9643,10 +9643,10 @@
       <x:c r="C129" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D129" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E129" s="4" t="n">
+      <x:c r="D129" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E129" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F129" s="4">
@@ -9706,10 +9706,10 @@
       <x:c r="C130" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D130" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E130" s="4" t="n">
+      <x:c r="D130" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E130" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F130" s="4">
@@ -9769,10 +9769,10 @@
       <x:c r="C131" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D131" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E131" s="4" t="n">
+      <x:c r="D131" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E131" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F131" s="4">
@@ -9832,10 +9832,10 @@
       <x:c r="C132" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D132" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E132" s="4" t="n">
+      <x:c r="D132" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E132" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F132" s="4">
@@ -9895,10 +9895,10 @@
       <x:c r="C133" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D133" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E133" s="4" t="n">
+      <x:c r="D133" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E133" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F133" s="4">
@@ -9958,19 +9958,19 @@
       <x:c r="C134" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D134" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E134" s="4" t="n">
-        <x:v>0</x:v>
+      <x:c r="D134" s="4">
+        <x:v>1165.4297928000001</x:v>
+      </x:c>
+      <x:c r="E134" s="4">
+        <x:v>135.51824994</x:v>
       </x:c>
       <x:c r="F134" s="4" t="n">
         <x:f>E134/7*5</x:f>
-        <x:v>0</x:v>
+        <x:v>96.79874995714286</x:v>
       </x:c>
       <x:c r="G134" s="4" t="n">
         <x:f>F134+E134</x:f>
-        <x:v>0</x:v>
+        <x:v>232.31699989714286</x:v>
       </x:c>
       <x:c r="H134" s="2">
         <x:v>0</x:v>
@@ -10023,10 +10023,10 @@
       <x:c r="C135" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D135" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E135" s="4" t="n">
+      <x:c r="D135" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E135" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F135" s="4">
@@ -10086,10 +10086,10 @@
       <x:c r="C136" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D136" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E136" s="4" t="n">
+      <x:c r="D136" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E136" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F136" s="4">
@@ -10149,10 +10149,10 @@
       <x:c r="C137" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D137" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E137" s="4" t="n">
+      <x:c r="D137" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E137" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F137" s="4">
@@ -10212,10 +10212,10 @@
       <x:c r="C138" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D138" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E138" s="4" t="n">
+      <x:c r="D138" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E138" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F138" s="4">
@@ -10275,10 +10275,10 @@
       <x:c r="C139" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D139" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E139" s="4" t="n">
+      <x:c r="D139" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E139" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F139" s="4">
@@ -10338,10 +10338,10 @@
       <x:c r="C140" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D140" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E140" s="4" t="n">
+      <x:c r="D140" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E140" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F140" s="4">
@@ -10401,10 +10401,10 @@
       <x:c r="C141" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D141" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E141" s="4" t="n">
+      <x:c r="D141" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E141" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F141" s="4">
@@ -10464,10 +10464,10 @@
       <x:c r="C142" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D142" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E142" s="4" t="n">
+      <x:c r="D142" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E142" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F142" s="4">
@@ -10527,10 +10527,10 @@
       <x:c r="C143" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D143" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E143" s="4" t="n">
+      <x:c r="D143" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E143" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F143" s="4">
@@ -10590,10 +10590,10 @@
       <x:c r="C144" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D144" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E144" s="4" t="n">
+      <x:c r="D144" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E144" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F144" s="4">
@@ -10653,10 +10653,10 @@
       <x:c r="C145" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D145" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E145" s="4" t="n">
+      <x:c r="D145" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E145" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F145" s="4">
@@ -10716,10 +10716,10 @@
       <x:c r="C146" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D146" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E146" s="4" t="n">
+      <x:c r="D146" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E146" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F146" s="4">
@@ -10779,10 +10779,10 @@
       <x:c r="C147" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D147" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E147" s="4" t="n">
+      <x:c r="D147" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E147" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F147" s="4">
@@ -10842,10 +10842,10 @@
       <x:c r="C148" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D148" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E148" s="4" t="n">
+      <x:c r="D148" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E148" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F148" s="4">
@@ -10905,10 +10905,10 @@
       <x:c r="C149" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D149" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E149" s="4" t="n">
+      <x:c r="D149" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E149" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F149" s="4">
@@ -10968,10 +10968,10 @@
       <x:c r="C150" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D150" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E150" s="4" t="n">
+      <x:c r="D150" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E150" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F150" s="4">
@@ -11031,10 +11031,10 @@
       <x:c r="C151" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D151" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E151" s="4" t="n">
+      <x:c r="D151" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E151" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F151" s="4">
@@ -11094,10 +11094,10 @@
       <x:c r="C152" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D152" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E152" s="4" t="n">
+      <x:c r="D152" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E152" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F152" s="4">
@@ -11157,10 +11157,10 @@
       <x:c r="C153" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D153" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E153" s="4" t="n">
+      <x:c r="D153" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E153" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F153" s="4">
@@ -11220,10 +11220,10 @@
       <x:c r="C154" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D154" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E154" s="4" t="n">
+      <x:c r="D154" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E154" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F154" s="4">
@@ -11283,10 +11283,10 @@
       <x:c r="C155" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D155" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E155" s="4" t="n">
+      <x:c r="D155" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E155" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F155" s="4">
@@ -11346,10 +11346,10 @@
       <x:c r="C156" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D156" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E156" s="4" t="n">
+      <x:c r="D156" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E156" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F156" s="4">
@@ -11409,10 +11409,10 @@
       <x:c r="C157" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D157" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E157" s="4" t="n">
+      <x:c r="D157" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E157" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F157" s="4">
@@ -11472,10 +11472,10 @@
       <x:c r="C158" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D158" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E158" s="4" t="n">
+      <x:c r="D158" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E158" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F158" s="4">
@@ -11535,19 +11535,19 @@
       <x:c r="C159" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D159" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E159" s="4" t="n">
-        <x:v>0</x:v>
+      <x:c r="D159" s="4">
+        <x:v>202.86490769999997</x:v>
+      </x:c>
+      <x:c r="E159" s="4">
+        <x:v>97.597140300000007</x:v>
       </x:c>
       <x:c r="F159" s="4" t="n">
         <x:f>E159/7*5</x:f>
-        <x:v>0</x:v>
+        <x:v>69.71224307142857</x:v>
       </x:c>
       <x:c r="G159" s="4" t="n">
         <x:f>F159+E159</x:f>
-        <x:v>0</x:v>
+        <x:v>167.30938337142857</x:v>
       </x:c>
       <x:c r="H159" s="2">
         <x:v>0</x:v>
@@ -11600,10 +11600,10 @@
       <x:c r="C160" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D160" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E160" s="4" t="n">
+      <x:c r="D160" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E160" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F160" s="4">
@@ -11663,19 +11663,19 @@
       <x:c r="C161" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D161" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E161" s="4" t="n">
-        <x:v>0</x:v>
+      <x:c r="D161" s="4">
+        <x:v>94.577301000000006</x:v>
+      </x:c>
+      <x:c r="E161" s="4">
+        <x:v>60.152633219999998</x:v>
       </x:c>
       <x:c r="F161" s="4" t="n">
         <x:f>E161/7*5</x:f>
-        <x:v>0</x:v>
+        <x:v>42.96616658571429</x:v>
       </x:c>
       <x:c r="G161" s="4" t="n">
         <x:f>F161+E161</x:f>
-        <x:v>0</x:v>
+        <x:v>103.11879980571429</x:v>
       </x:c>
       <x:c r="H161" s="2">
         <x:v>0</x:v>
@@ -11728,10 +11728,10 @@
       <x:c r="C162" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D162" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E162" s="4" t="n">
+      <x:c r="D162" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E162" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F162" s="4">
@@ -11791,10 +11791,10 @@
       <x:c r="C163" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D163" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E163" s="4" t="n">
+      <x:c r="D163" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E163" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F163" s="4">
@@ -11854,10 +11854,10 @@
       <x:c r="C164" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D164" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E164" s="4" t="n">
+      <x:c r="D164" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E164" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F164" s="4">
@@ -11917,10 +11917,10 @@
       <x:c r="C165" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D165" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E165" s="4" t="n">
+      <x:c r="D165" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E165" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F165" s="4">
@@ -11980,10 +11980,10 @@
       <x:c r="C166" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D166" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E166" s="4" t="n">
+      <x:c r="D166" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E166" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F166" s="4">
@@ -12043,10 +12043,10 @@
       <x:c r="C167" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D167" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E167" s="4" t="n">
+      <x:c r="D167" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E167" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F167" s="4">
@@ -12106,10 +12106,10 @@
       <x:c r="C168" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D168" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E168" s="4" t="n">
+      <x:c r="D168" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E168" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F168" s="4">
@@ -12169,10 +12169,10 @@
       <x:c r="C169" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D169" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E169" s="4" t="n">
+      <x:c r="D169" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E169" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F169" s="4">
@@ -12232,10 +12232,10 @@
       <x:c r="C170" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D170" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E170" s="4" t="n">
+      <x:c r="D170" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E170" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F170" s="4">
@@ -12295,10 +12295,10 @@
       <x:c r="C171" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D171" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E171" s="4" t="n">
+      <x:c r="D171" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E171" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F171" s="4">
@@ -12358,10 +12358,10 @@
       <x:c r="C172" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D172" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E172" s="4" t="n">
+      <x:c r="D172" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E172" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F172" s="4">
@@ -12421,10 +12421,10 @@
       <x:c r="C173" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D173" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E173" s="4" t="n">
+      <x:c r="D173" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E173" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F173" s="4">
@@ -12484,10 +12484,10 @@
       <x:c r="C174" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D174" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E174" s="4" t="n">
+      <x:c r="D174" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E174" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F174" s="4">
@@ -12547,10 +12547,10 @@
       <x:c r="C175" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D175" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E175" s="4" t="n">
+      <x:c r="D175" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E175" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F175" s="4">
@@ -12610,19 +12610,19 @@
       <x:c r="C176" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D176" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E176" s="4" t="n">
-        <x:v>0</x:v>
+      <x:c r="D176" s="4">
+        <x:v>1253.4134885999997</x:v>
+      </x:c>
+      <x:c r="E176" s="4">
+        <x:v>921.60064914999998</x:v>
       </x:c>
       <x:c r="F176" s="4" t="n">
         <x:f>E176/7*5</x:f>
-        <x:v>0</x:v>
+        <x:v>658.2861779642858</x:v>
       </x:c>
       <x:c r="G176" s="4" t="n">
         <x:f>F176+E176</x:f>
-        <x:v>0</x:v>
+        <x:v>1579.8868271142858</x:v>
       </x:c>
       <x:c r="H176" s="2">
         <x:v>0</x:v>
@@ -12675,10 +12675,10 @@
       <x:c r="C177" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D177" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E177" s="4" t="n">
+      <x:c r="D177" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E177" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F177" s="4">
@@ -12734,19 +12734,19 @@
       </x:c>
       <x:c r="D178" s="6" t="n">
         <x:f>SUM(D2:D177)</x:f>
-        <x:v>0</x:v>
+        <x:v>32331.7340073</x:v>
       </x:c>
       <x:c r="E178" s="6" t="n">
         <x:f>SUM(E2:E177)</x:f>
-        <x:v>0</x:v>
+        <x:v>16381.042992609999</x:v>
       </x:c>
       <x:c r="F178" s="6" t="n">
         <x:f>SUM(F2:F177)</x:f>
-        <x:v>0</x:v>
+        <x:v>11700.744994721428</x:v>
       </x:c>
       <x:c r="G178" s="6" t="n">
         <x:f>SUM(G2:G177)</x:f>
-        <x:v>0</x:v>
+        <x:v>28081.78798733143</x:v>
       </x:c>
       <x:c r="T178" s="8" t="n">
         <x:f>SUM(T2:T177)</x:f>

</xml_diff>

<commit_message>
Show Tunis Landing values (#12)
Restore the supplied Landing references in the Tunis workbook and display Landing beside FY Budget 2027 throughout the Tunis OPEX page.
</commit_message>
<xml_diff>
--- a/templates/Tunis_OPEX_2027.xlsx
+++ b/templates/Tunis_OPEX_2027.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tunis OPEX 2027" sheetId="2" r:id="Re54122d4af8f4af3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tunis OPEX 2027" sheetId="2" r:id="R988e6bdba4e74b57"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1638,19 +1638,19 @@
       <x:c r="C2" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D2" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E2" s="4" t="n">
-        <x:v>0</x:v>
+      <x:c r="D2" s="4">
+        <x:v>25651.324717200001</x:v>
+      </x:c>
+      <x:c r="E2" s="4">
+        <x:v>14314.6255</x:v>
       </x:c>
       <x:c r="F2" s="4" t="n">
         <x:f>E2/7*5</x:f>
-        <x:v>0</x:v>
+        <x:v>10224.7325</x:v>
       </x:c>
       <x:c r="G2" s="4" t="n">
         <x:f>F2+E2</x:f>
-        <x:v>0</x:v>
+        <x:v>24539.358</x:v>
       </x:c>
       <x:c r="H2" s="2">
         <x:v>0</x:v>
@@ -1703,10 +1703,10 @@
       <x:c r="C3" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D3" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E3" s="4" t="n">
+      <x:c r="D3" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E3" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F3" s="4">
@@ -1766,10 +1766,10 @@
       <x:c r="C4" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D4" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E4" s="4" t="n">
+      <x:c r="D4" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E4" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F4" s="4">
@@ -1829,10 +1829,10 @@
       <x:c r="C5" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D5" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E5" s="4" t="n">
+      <x:c r="D5" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E5" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F5" s="4">
@@ -1892,10 +1892,10 @@
       <x:c r="C6" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D6" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E6" s="4" t="n">
+      <x:c r="D6" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E6" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F6" s="4">
@@ -1955,10 +1955,10 @@
       <x:c r="C7" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D7" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E7" s="4" t="n">
+      <x:c r="D7" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E7" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F7" s="4">
@@ -2018,10 +2018,10 @@
       <x:c r="C8" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D8" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E8" s="4" t="n">
+      <x:c r="D8" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E8" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F8" s="4">
@@ -2081,10 +2081,10 @@
       <x:c r="C9" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D9" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E9" s="4" t="n">
+      <x:c r="D9" s="4">
+        <x:v>98.28</x:v>
+      </x:c>
+      <x:c r="E9" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F9" s="4">
@@ -2144,10 +2144,10 @@
       <x:c r="C10" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D10" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E10" s="4" t="n">
+      <x:c r="D10" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E10" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F10" s="4">
@@ -2207,10 +2207,10 @@
       <x:c r="C11" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D11" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E11" s="4" t="n">
+      <x:c r="D11" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E11" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F11" s="4">
@@ -2270,10 +2270,10 @@
       <x:c r="C12" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D12" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E12" s="4" t="n">
+      <x:c r="D12" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E12" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F12" s="4">
@@ -2333,10 +2333,10 @@
       <x:c r="C13" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D13" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E13" s="4" t="n">
+      <x:c r="D13" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E13" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F13" s="4">
@@ -2396,10 +2396,10 @@
       <x:c r="C14" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D14" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E14" s="4" t="n">
+      <x:c r="D14" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E14" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F14" s="4">
@@ -2459,10 +2459,10 @@
       <x:c r="C15" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D15" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E15" s="4" t="n">
+      <x:c r="D15" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E15" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F15" s="4">
@@ -2522,10 +2522,10 @@
       <x:c r="C16" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D16" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E16" s="4" t="n">
+      <x:c r="D16" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E16" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F16" s="4">
@@ -2585,10 +2585,10 @@
       <x:c r="C17" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D17" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E17" s="4" t="n">
+      <x:c r="D17" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E17" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F17" s="4">
@@ -2648,10 +2648,10 @@
       <x:c r="C18" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D18" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E18" s="4" t="n">
+      <x:c r="D18" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E18" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F18" s="4">
@@ -2711,10 +2711,10 @@
       <x:c r="C19" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D19" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E19" s="4" t="n">
+      <x:c r="D19" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E19" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F19" s="4">
@@ -2774,10 +2774,10 @@
       <x:c r="C20" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D20" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E20" s="4" t="n">
+      <x:c r="D20" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E20" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F20" s="4">
@@ -2837,10 +2837,10 @@
       <x:c r="C21" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D21" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E21" s="4" t="n">
+      <x:c r="D21" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E21" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F21" s="4">
@@ -2900,10 +2900,10 @@
       <x:c r="C22" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D22" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E22" s="4" t="n">
+      <x:c r="D22" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E22" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F22" s="4">
@@ -2963,10 +2963,10 @@
       <x:c r="C23" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D23" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E23" s="4" t="n">
+      <x:c r="D23" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E23" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F23" s="4">
@@ -3026,10 +3026,10 @@
       <x:c r="C24" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D24" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E24" s="4" t="n">
+      <x:c r="D24" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E24" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F24" s="4">
@@ -3089,10 +3089,10 @@
       <x:c r="C25" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D25" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E25" s="4" t="n">
+      <x:c r="D25" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E25" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F25" s="4">
@@ -3152,10 +3152,10 @@
       <x:c r="C26" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D26" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E26" s="4" t="n">
+      <x:c r="D26" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E26" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F26" s="4">
@@ -3215,10 +3215,10 @@
       <x:c r="C27" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D27" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E27" s="4" t="n">
+      <x:c r="D27" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E27" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F27" s="4">
@@ -3278,10 +3278,10 @@
       <x:c r="C28" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D28" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E28" s="4" t="n">
+      <x:c r="D28" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E28" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F28" s="4">
@@ -3341,10 +3341,10 @@
       <x:c r="C29" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D29" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E29" s="4" t="n">
+      <x:c r="D29" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E29" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F29" s="4">
@@ -3404,10 +3404,10 @@
       <x:c r="C30" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D30" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E30" s="4" t="n">
+      <x:c r="D30" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E30" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F30" s="4">
@@ -3467,10 +3467,10 @@
       <x:c r="C31" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D31" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E31" s="4" t="n">
+      <x:c r="D31" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E31" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F31" s="4">
@@ -3530,10 +3530,10 @@
       <x:c r="C32" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D32" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E32" s="4" t="n">
+      <x:c r="D32" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E32" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F32" s="4">
@@ -3593,10 +3593,10 @@
       <x:c r="C33" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D33" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E33" s="4" t="n">
+      <x:c r="D33" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E33" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F33" s="4">
@@ -3656,10 +3656,10 @@
       <x:c r="C34" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D34" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E34" s="4" t="n">
+      <x:c r="D34" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E34" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F34" s="4">
@@ -3719,10 +3719,10 @@
       <x:c r="C35" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D35" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E35" s="4" t="n">
+      <x:c r="D35" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E35" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F35" s="4">
@@ -3782,10 +3782,10 @@
       <x:c r="C36" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D36" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E36" s="4" t="n">
+      <x:c r="D36" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E36" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F36" s="4">
@@ -3845,10 +3845,10 @@
       <x:c r="C37" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D37" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E37" s="4" t="n">
+      <x:c r="D37" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E37" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F37" s="4">
@@ -3908,10 +3908,10 @@
       <x:c r="C38" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D38" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E38" s="4" t="n">
+      <x:c r="D38" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E38" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F38" s="4">
@@ -3971,10 +3971,10 @@
       <x:c r="C39" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D39" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E39" s="4" t="n">
+      <x:c r="D39" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E39" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F39" s="4">
@@ -4034,10 +4034,10 @@
       <x:c r="C40" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D40" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E40" s="4" t="n">
+      <x:c r="D40" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E40" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F40" s="4">
@@ -4097,10 +4097,10 @@
       <x:c r="C41" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D41" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E41" s="4" t="n">
+      <x:c r="D41" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E41" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F41" s="4">
@@ -4160,10 +4160,10 @@
       <x:c r="C42" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D42" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E42" s="4" t="n">
+      <x:c r="D42" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E42" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F42" s="4">
@@ -4223,10 +4223,10 @@
       <x:c r="C43" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D43" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E43" s="4" t="n">
+      <x:c r="D43" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E43" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F43" s="4">
@@ -4286,10 +4286,10 @@
       <x:c r="C44" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D44" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E44" s="4" t="n">
+      <x:c r="D44" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E44" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F44" s="4">
@@ -4349,10 +4349,10 @@
       <x:c r="C45" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D45" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E45" s="4" t="n">
+      <x:c r="D45" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E45" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F45" s="4">
@@ -4412,10 +4412,10 @@
       <x:c r="C46" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D46" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E46" s="4" t="n">
+      <x:c r="D46" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E46" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F46" s="4">
@@ -4475,10 +4475,10 @@
       <x:c r="C47" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D47" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E47" s="4" t="n">
+      <x:c r="D47" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E47" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F47" s="4">
@@ -4538,10 +4538,10 @@
       <x:c r="C48" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D48" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E48" s="4" t="n">
+      <x:c r="D48" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E48" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F48" s="4">
@@ -4601,10 +4601,10 @@
       <x:c r="C49" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D49" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E49" s="4" t="n">
+      <x:c r="D49" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E49" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F49" s="4">
@@ -4664,10 +4664,10 @@
       <x:c r="C50" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D50" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E50" s="4" t="n">
+      <x:c r="D50" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E50" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F50" s="4">
@@ -4727,10 +4727,10 @@
       <x:c r="C51" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D51" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E51" s="4" t="n">
+      <x:c r="D51" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E51" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F51" s="4">
@@ -4790,10 +4790,10 @@
       <x:c r="C52" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D52" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E52" s="4" t="n">
+      <x:c r="D52" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E52" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F52" s="4">
@@ -4853,10 +4853,10 @@
       <x:c r="C53" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D53" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E53" s="4" t="n">
+      <x:c r="D53" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E53" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F53" s="4">
@@ -4916,10 +4916,10 @@
       <x:c r="C54" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D54" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E54" s="4" t="n">
+      <x:c r="D54" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E54" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F54" s="4">
@@ -4979,10 +4979,10 @@
       <x:c r="C55" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D55" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E55" s="4" t="n">
+      <x:c r="D55" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E55" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F55" s="4">
@@ -5042,10 +5042,10 @@
       <x:c r="C56" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D56" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E56" s="4" t="n">
+      <x:c r="D56" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E56" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F56" s="4">
@@ -5105,10 +5105,10 @@
       <x:c r="C57" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D57" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E57" s="4" t="n">
+      <x:c r="D57" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E57" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F57" s="4">
@@ -5168,10 +5168,10 @@
       <x:c r="C58" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D58" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E58" s="4" t="n">
+      <x:c r="D58" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E58" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F58" s="4">
@@ -5231,10 +5231,10 @@
       <x:c r="C59" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D59" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E59" s="4" t="n">
+      <x:c r="D59" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E59" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F59" s="4">
@@ -5294,10 +5294,10 @@
       <x:c r="C60" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D60" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E60" s="4" t="n">
+      <x:c r="D60" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E60" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F60" s="4">
@@ -5357,10 +5357,10 @@
       <x:c r="C61" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D61" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E61" s="4" t="n">
+      <x:c r="D61" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E61" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F61" s="4">
@@ -5420,10 +5420,10 @@
       <x:c r="C62" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D62" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E62" s="4" t="n">
+      <x:c r="D62" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E62" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F62" s="4">
@@ -5483,10 +5483,10 @@
       <x:c r="C63" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D63" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E63" s="4" t="n">
+      <x:c r="D63" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E63" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F63" s="4">
@@ -5546,10 +5546,10 @@
       <x:c r="C64" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D64" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E64" s="4" t="n">
+      <x:c r="D64" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E64" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F64" s="4">
@@ -5609,10 +5609,10 @@
       <x:c r="C65" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D65" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E65" s="4" t="n">
+      <x:c r="D65" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E65" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F65" s="4">
@@ -5672,10 +5672,10 @@
       <x:c r="C66" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D66" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E66" s="4" t="n">
+      <x:c r="D66" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E66" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F66" s="4">
@@ -5735,10 +5735,10 @@
       <x:c r="C67" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D67" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E67" s="4" t="n">
+      <x:c r="D67" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E67" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F67" s="4">
@@ -5798,10 +5798,10 @@
       <x:c r="C68" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D68" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E68" s="4" t="n">
+      <x:c r="D68" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E68" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F68" s="4">
@@ -5861,10 +5861,10 @@
       <x:c r="C69" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D69" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E69" s="4" t="n">
+      <x:c r="D69" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E69" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F69" s="4">
@@ -5924,10 +5924,10 @@
       <x:c r="C70" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D70" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E70" s="4" t="n">
+      <x:c r="D70" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E70" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F70" s="4">
@@ -5987,10 +5987,10 @@
       <x:c r="C71" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D71" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E71" s="4" t="n">
+      <x:c r="D71" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E71" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F71" s="4">
@@ -6050,10 +6050,10 @@
       <x:c r="C72" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D72" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E72" s="4" t="n">
+      <x:c r="D72" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E72" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F72" s="4">
@@ -6113,10 +6113,10 @@
       <x:c r="C73" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D73" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E73" s="4" t="n">
+      <x:c r="D73" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E73" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F73" s="4">
@@ -6176,10 +6176,10 @@
       <x:c r="C74" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D74" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E74" s="4" t="n">
+      <x:c r="D74" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E74" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F74" s="4">
@@ -6239,10 +6239,10 @@
       <x:c r="C75" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D75" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E75" s="4" t="n">
+      <x:c r="D75" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E75" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F75" s="4">
@@ -6302,10 +6302,10 @@
       <x:c r="C76" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D76" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E76" s="4" t="n">
+      <x:c r="D76" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E76" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F76" s="4">
@@ -6365,10 +6365,10 @@
       <x:c r="C77" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D77" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E77" s="4" t="n">
+      <x:c r="D77" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E77" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F77" s="4">
@@ -6428,10 +6428,10 @@
       <x:c r="C78" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D78" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E78" s="4" t="n">
+      <x:c r="D78" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E78" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F78" s="4">
@@ -6491,10 +6491,10 @@
       <x:c r="C79" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D79" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E79" s="4" t="n">
+      <x:c r="D79" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E79" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F79" s="4">
@@ -6554,10 +6554,10 @@
       <x:c r="C80" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D80" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E80" s="4" t="n">
+      <x:c r="D80" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E80" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F80" s="4">
@@ -6617,10 +6617,10 @@
       <x:c r="C81" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D81" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E81" s="4" t="n">
+      <x:c r="D81" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E81" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F81" s="4">
@@ -6680,10 +6680,10 @@
       <x:c r="C82" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D82" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E82" s="4" t="n">
+      <x:c r="D82" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E82" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F82" s="4">
@@ -6743,10 +6743,10 @@
       <x:c r="C83" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D83" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E83" s="4" t="n">
+      <x:c r="D83" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E83" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F83" s="4">
@@ -6806,10 +6806,10 @@
       <x:c r="C84" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D84" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E84" s="4" t="n">
+      <x:c r="D84" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E84" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F84" s="4">
@@ -6869,10 +6869,10 @@
       <x:c r="C85" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D85" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E85" s="4" t="n">
+      <x:c r="D85" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E85" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F85" s="4">
@@ -6932,10 +6932,10 @@
       <x:c r="C86" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D86" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E86" s="4" t="n">
+      <x:c r="D86" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E86" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F86" s="4">
@@ -6995,10 +6995,10 @@
       <x:c r="C87" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D87" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E87" s="4" t="n">
+      <x:c r="D87" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E87" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F87" s="4">
@@ -7058,10 +7058,10 @@
       <x:c r="C88" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D88" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E88" s="4" t="n">
+      <x:c r="D88" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E88" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F88" s="4">
@@ -7121,10 +7121,10 @@
       <x:c r="C89" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D89" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E89" s="4" t="n">
+      <x:c r="D89" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E89" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F89" s="4">
@@ -7184,10 +7184,10 @@
       <x:c r="C90" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D90" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E90" s="4" t="n">
+      <x:c r="D90" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E90" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F90" s="4">
@@ -7247,10 +7247,10 @@
       <x:c r="C91" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D91" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E91" s="4" t="n">
+      <x:c r="D91" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E91" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F91" s="4">
@@ -7310,10 +7310,10 @@
       <x:c r="C92" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D92" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E92" s="4" t="n">
+      <x:c r="D92" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E92" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F92" s="4">
@@ -7373,10 +7373,10 @@
       <x:c r="C93" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D93" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E93" s="4" t="n">
+      <x:c r="D93" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E93" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F93" s="4">
@@ -7436,10 +7436,10 @@
       <x:c r="C94" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D94" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E94" s="4" t="n">
+      <x:c r="D94" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E94" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F94" s="4">
@@ -7499,10 +7499,10 @@
       <x:c r="C95" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D95" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E95" s="4" t="n">
+      <x:c r="D95" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E95" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F95" s="4">
@@ -7562,10 +7562,10 @@
       <x:c r="C96" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D96" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E96" s="4" t="n">
+      <x:c r="D96" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E96" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F96" s="4">
@@ -7625,10 +7625,10 @@
       <x:c r="C97" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D97" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E97" s="4" t="n">
+      <x:c r="D97" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E97" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F97" s="4">
@@ -7688,10 +7688,10 @@
       <x:c r="C98" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D98" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E98" s="4" t="n">
+      <x:c r="D98" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E98" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F98" s="4">
@@ -7751,10 +7751,10 @@
       <x:c r="C99" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D99" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E99" s="4" t="n">
+      <x:c r="D99" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E99" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F99" s="4">
@@ -7814,10 +7814,10 @@
       <x:c r="C100" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D100" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E100" s="4" t="n">
+      <x:c r="D100" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E100" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F100" s="4">
@@ -7877,10 +7877,10 @@
       <x:c r="C101" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D101" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E101" s="4" t="n">
+      <x:c r="D101" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E101" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F101" s="4">
@@ -7940,10 +7940,10 @@
       <x:c r="C102" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D102" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E102" s="4" t="n">
+      <x:c r="D102" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E102" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F102" s="4">
@@ -8003,10 +8003,10 @@
       <x:c r="C103" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D103" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E103" s="4" t="n">
+      <x:c r="D103" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E103" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F103" s="4">
@@ -8066,10 +8066,10 @@
       <x:c r="C104" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D104" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E104" s="4" t="n">
+      <x:c r="D104" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E104" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F104" s="4">
@@ -8129,10 +8129,10 @@
       <x:c r="C105" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D105" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E105" s="4" t="n">
+      <x:c r="D105" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E105" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F105" s="4">
@@ -8192,10 +8192,10 @@
       <x:c r="C106" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D106" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E106" s="4" t="n">
+      <x:c r="D106" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E106" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F106" s="4">
@@ -8255,19 +8255,19 @@
       <x:c r="C107" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D107" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E107" s="4" t="n">
-        <x:v>0</x:v>
+      <x:c r="D107" s="4">
+        <x:v>3865.8438000000001</x:v>
+      </x:c>
+      <x:c r="E107" s="4">
+        <x:v>851.54881999999998</x:v>
       </x:c>
       <x:c r="F107" s="4" t="n">
         <x:f>E107/7*5</x:f>
-        <x:v>0</x:v>
+        <x:v>608.2491571428571</x:v>
       </x:c>
       <x:c r="G107" s="4" t="n">
         <x:f>F107+E107</x:f>
-        <x:v>0</x:v>
+        <x:v>1459.7979771428572</x:v>
       </x:c>
       <x:c r="H107" s="2">
         <x:v>0</x:v>
@@ -8320,10 +8320,10 @@
       <x:c r="C108" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D108" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E108" s="4" t="n">
+      <x:c r="D108" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E108" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F108" s="4">
@@ -8383,10 +8383,10 @@
       <x:c r="C109" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D109" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E109" s="4" t="n">
+      <x:c r="D109" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E109" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F109" s="4">
@@ -8446,10 +8446,10 @@
       <x:c r="C110" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D110" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E110" s="4" t="n">
+      <x:c r="D110" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E110" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F110" s="4">
@@ -8509,10 +8509,10 @@
       <x:c r="C111" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D111" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E111" s="4" t="n">
+      <x:c r="D111" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E111" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F111" s="4">
@@ -8572,10 +8572,10 @@
       <x:c r="C112" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D112" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E112" s="4" t="n">
+      <x:c r="D112" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E112" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F112" s="4">
@@ -8635,10 +8635,10 @@
       <x:c r="C113" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D113" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E113" s="4" t="n">
+      <x:c r="D113" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E113" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F113" s="4">
@@ -8698,10 +8698,10 @@
       <x:c r="C114" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D114" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E114" s="4" t="n">
+      <x:c r="D114" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E114" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F114" s="4">
@@ -8761,10 +8761,10 @@
       <x:c r="C115" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D115" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E115" s="4" t="n">
+      <x:c r="D115" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E115" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F115" s="4">
@@ -8824,10 +8824,10 @@
       <x:c r="C116" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D116" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E116" s="4" t="n">
+      <x:c r="D116" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E116" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F116" s="4">
@@ -8887,10 +8887,10 @@
       <x:c r="C117" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D117" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E117" s="4" t="n">
+      <x:c r="D117" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E117" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F117" s="4">
@@ -8950,10 +8950,10 @@
       <x:c r="C118" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D118" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E118" s="4" t="n">
+      <x:c r="D118" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E118" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F118" s="4">
@@ -9013,10 +9013,10 @@
       <x:c r="C119" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D119" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E119" s="4" t="n">
+      <x:c r="D119" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E119" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F119" s="4">
@@ -9076,10 +9076,10 @@
       <x:c r="C120" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D120" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E120" s="4" t="n">
+      <x:c r="D120" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E120" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F120" s="4">
@@ -9139,10 +9139,10 @@
       <x:c r="C121" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D121" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E121" s="4" t="n">
+      <x:c r="D121" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E121" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F121" s="4">
@@ -9202,10 +9202,10 @@
       <x:c r="C122" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D122" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E122" s="4" t="n">
+      <x:c r="D122" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E122" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F122" s="4">
@@ -9265,10 +9265,10 @@
       <x:c r="C123" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D123" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E123" s="4" t="n">
+      <x:c r="D123" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E123" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F123" s="4">
@@ -9328,10 +9328,10 @@
       <x:c r="C124" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D124" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E124" s="4" t="n">
+      <x:c r="D124" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E124" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F124" s="4">
@@ -9391,10 +9391,10 @@
       <x:c r="C125" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D125" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E125" s="4" t="n">
+      <x:c r="D125" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E125" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F125" s="4">
@@ -9454,10 +9454,10 @@
       <x:c r="C126" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D126" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E126" s="4" t="n">
+      <x:c r="D126" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E126" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F126" s="4">
@@ -9517,10 +9517,10 @@
       <x:c r="C127" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D127" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E127" s="4" t="n">
+      <x:c r="D127" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E127" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F127" s="4">
@@ -9580,10 +9580,10 @@
       <x:c r="C128" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D128" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E128" s="4" t="n">
+      <x:c r="D128" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E128" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F128" s="4">
@@ -9643,10 +9643,10 @@
       <x:c r="C129" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D129" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E129" s="4" t="n">
+      <x:c r="D129" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E129" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F129" s="4">
@@ -9706,10 +9706,10 @@
       <x:c r="C130" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D130" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E130" s="4" t="n">
+      <x:c r="D130" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E130" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F130" s="4">
@@ -9769,10 +9769,10 @@
       <x:c r="C131" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D131" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E131" s="4" t="n">
+      <x:c r="D131" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E131" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F131" s="4">
@@ -9832,10 +9832,10 @@
       <x:c r="C132" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D132" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E132" s="4" t="n">
+      <x:c r="D132" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E132" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F132" s="4">
@@ -9895,10 +9895,10 @@
       <x:c r="C133" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D133" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E133" s="4" t="n">
+      <x:c r="D133" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E133" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F133" s="4">
@@ -9958,19 +9958,19 @@
       <x:c r="C134" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D134" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E134" s="4" t="n">
-        <x:v>0</x:v>
+      <x:c r="D134" s="4">
+        <x:v>1165.4297928000001</x:v>
+      </x:c>
+      <x:c r="E134" s="4">
+        <x:v>135.51824994</x:v>
       </x:c>
       <x:c r="F134" s="4" t="n">
         <x:f>E134/7*5</x:f>
-        <x:v>0</x:v>
+        <x:v>96.79874995714286</x:v>
       </x:c>
       <x:c r="G134" s="4" t="n">
         <x:f>F134+E134</x:f>
-        <x:v>0</x:v>
+        <x:v>232.31699989714286</x:v>
       </x:c>
       <x:c r="H134" s="2">
         <x:v>0</x:v>
@@ -10023,10 +10023,10 @@
       <x:c r="C135" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D135" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E135" s="4" t="n">
+      <x:c r="D135" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E135" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F135" s="4">
@@ -10086,10 +10086,10 @@
       <x:c r="C136" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D136" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E136" s="4" t="n">
+      <x:c r="D136" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E136" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F136" s="4">
@@ -10149,10 +10149,10 @@
       <x:c r="C137" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D137" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E137" s="4" t="n">
+      <x:c r="D137" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E137" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F137" s="4">
@@ -10212,10 +10212,10 @@
       <x:c r="C138" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D138" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E138" s="4" t="n">
+      <x:c r="D138" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E138" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F138" s="4">
@@ -10275,10 +10275,10 @@
       <x:c r="C139" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D139" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E139" s="4" t="n">
+      <x:c r="D139" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E139" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F139" s="4">
@@ -10338,10 +10338,10 @@
       <x:c r="C140" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D140" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E140" s="4" t="n">
+      <x:c r="D140" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E140" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F140" s="4">
@@ -10401,10 +10401,10 @@
       <x:c r="C141" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D141" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E141" s="4" t="n">
+      <x:c r="D141" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E141" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F141" s="4">
@@ -10464,10 +10464,10 @@
       <x:c r="C142" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D142" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E142" s="4" t="n">
+      <x:c r="D142" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E142" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F142" s="4">
@@ -10527,10 +10527,10 @@
       <x:c r="C143" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D143" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E143" s="4" t="n">
+      <x:c r="D143" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E143" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F143" s="4">
@@ -10590,10 +10590,10 @@
       <x:c r="C144" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D144" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E144" s="4" t="n">
+      <x:c r="D144" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E144" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F144" s="4">
@@ -10653,10 +10653,10 @@
       <x:c r="C145" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D145" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E145" s="4" t="n">
+      <x:c r="D145" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E145" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F145" s="4">
@@ -10716,10 +10716,10 @@
       <x:c r="C146" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D146" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E146" s="4" t="n">
+      <x:c r="D146" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E146" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F146" s="4">
@@ -10779,10 +10779,10 @@
       <x:c r="C147" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D147" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E147" s="4" t="n">
+      <x:c r="D147" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E147" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F147" s="4">
@@ -10842,10 +10842,10 @@
       <x:c r="C148" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D148" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E148" s="4" t="n">
+      <x:c r="D148" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E148" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F148" s="4">
@@ -10905,10 +10905,10 @@
       <x:c r="C149" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D149" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E149" s="4" t="n">
+      <x:c r="D149" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E149" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F149" s="4">
@@ -10968,10 +10968,10 @@
       <x:c r="C150" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D150" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E150" s="4" t="n">
+      <x:c r="D150" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E150" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F150" s="4">
@@ -11031,10 +11031,10 @@
       <x:c r="C151" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D151" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E151" s="4" t="n">
+      <x:c r="D151" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E151" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F151" s="4">
@@ -11094,10 +11094,10 @@
       <x:c r="C152" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D152" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E152" s="4" t="n">
+      <x:c r="D152" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E152" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F152" s="4">
@@ -11157,10 +11157,10 @@
       <x:c r="C153" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D153" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E153" s="4" t="n">
+      <x:c r="D153" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E153" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F153" s="4">
@@ -11220,10 +11220,10 @@
       <x:c r="C154" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D154" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E154" s="4" t="n">
+      <x:c r="D154" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E154" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F154" s="4">
@@ -11283,10 +11283,10 @@
       <x:c r="C155" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D155" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E155" s="4" t="n">
+      <x:c r="D155" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E155" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F155" s="4">
@@ -11346,10 +11346,10 @@
       <x:c r="C156" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D156" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E156" s="4" t="n">
+      <x:c r="D156" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E156" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F156" s="4">
@@ -11409,10 +11409,10 @@
       <x:c r="C157" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D157" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E157" s="4" t="n">
+      <x:c r="D157" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E157" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F157" s="4">
@@ -11472,10 +11472,10 @@
       <x:c r="C158" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D158" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E158" s="4" t="n">
+      <x:c r="D158" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E158" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F158" s="4">
@@ -11535,19 +11535,19 @@
       <x:c r="C159" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D159" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E159" s="4" t="n">
-        <x:v>0</x:v>
+      <x:c r="D159" s="4">
+        <x:v>202.86490769999997</x:v>
+      </x:c>
+      <x:c r="E159" s="4">
+        <x:v>97.597140300000007</x:v>
       </x:c>
       <x:c r="F159" s="4" t="n">
         <x:f>E159/7*5</x:f>
-        <x:v>0</x:v>
+        <x:v>69.71224307142857</x:v>
       </x:c>
       <x:c r="G159" s="4" t="n">
         <x:f>F159+E159</x:f>
-        <x:v>0</x:v>
+        <x:v>167.30938337142857</x:v>
       </x:c>
       <x:c r="H159" s="2">
         <x:v>0</x:v>
@@ -11600,10 +11600,10 @@
       <x:c r="C160" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D160" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E160" s="4" t="n">
+      <x:c r="D160" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E160" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F160" s="4">
@@ -11663,19 +11663,19 @@
       <x:c r="C161" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D161" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E161" s="4" t="n">
-        <x:v>0</x:v>
+      <x:c r="D161" s="4">
+        <x:v>94.577301000000006</x:v>
+      </x:c>
+      <x:c r="E161" s="4">
+        <x:v>60.152633219999998</x:v>
       </x:c>
       <x:c r="F161" s="4" t="n">
         <x:f>E161/7*5</x:f>
-        <x:v>0</x:v>
+        <x:v>42.96616658571429</x:v>
       </x:c>
       <x:c r="G161" s="4" t="n">
         <x:f>F161+E161</x:f>
-        <x:v>0</x:v>
+        <x:v>103.11879980571429</x:v>
       </x:c>
       <x:c r="H161" s="2">
         <x:v>0</x:v>
@@ -11728,10 +11728,10 @@
       <x:c r="C162" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D162" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E162" s="4" t="n">
+      <x:c r="D162" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E162" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F162" s="4">
@@ -11791,10 +11791,10 @@
       <x:c r="C163" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D163" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E163" s="4" t="n">
+      <x:c r="D163" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E163" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F163" s="4">
@@ -11854,10 +11854,10 @@
       <x:c r="C164" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D164" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E164" s="4" t="n">
+      <x:c r="D164" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E164" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F164" s="4">
@@ -11917,10 +11917,10 @@
       <x:c r="C165" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D165" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E165" s="4" t="n">
+      <x:c r="D165" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E165" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F165" s="4">
@@ -11980,10 +11980,10 @@
       <x:c r="C166" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D166" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E166" s="4" t="n">
+      <x:c r="D166" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E166" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F166" s="4">
@@ -12043,10 +12043,10 @@
       <x:c r="C167" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D167" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E167" s="4" t="n">
+      <x:c r="D167" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E167" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F167" s="4">
@@ -12106,10 +12106,10 @@
       <x:c r="C168" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D168" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E168" s="4" t="n">
+      <x:c r="D168" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E168" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F168" s="4">
@@ -12169,10 +12169,10 @@
       <x:c r="C169" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D169" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E169" s="4" t="n">
+      <x:c r="D169" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E169" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F169" s="4">
@@ -12232,10 +12232,10 @@
       <x:c r="C170" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D170" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E170" s="4" t="n">
+      <x:c r="D170" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E170" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F170" s="4">
@@ -12295,10 +12295,10 @@
       <x:c r="C171" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D171" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E171" s="4" t="n">
+      <x:c r="D171" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E171" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F171" s="4">
@@ -12358,10 +12358,10 @@
       <x:c r="C172" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D172" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E172" s="4" t="n">
+      <x:c r="D172" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E172" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F172" s="4">
@@ -12421,10 +12421,10 @@
       <x:c r="C173" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D173" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E173" s="4" t="n">
+      <x:c r="D173" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E173" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F173" s="4">
@@ -12484,10 +12484,10 @@
       <x:c r="C174" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D174" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E174" s="4" t="n">
+      <x:c r="D174" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E174" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F174" s="4">
@@ -12547,10 +12547,10 @@
       <x:c r="C175" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D175" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E175" s="4" t="n">
+      <x:c r="D175" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E175" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F175" s="4">
@@ -12610,19 +12610,19 @@
       <x:c r="C176" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D176" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E176" s="4" t="n">
-        <x:v>0</x:v>
+      <x:c r="D176" s="4">
+        <x:v>1253.4134885999997</x:v>
+      </x:c>
+      <x:c r="E176" s="4">
+        <x:v>921.60064914999998</x:v>
       </x:c>
       <x:c r="F176" s="4" t="n">
         <x:f>E176/7*5</x:f>
-        <x:v>0</x:v>
+        <x:v>658.2861779642858</x:v>
       </x:c>
       <x:c r="G176" s="4" t="n">
         <x:f>F176+E176</x:f>
-        <x:v>0</x:v>
+        <x:v>1579.8868271142858</x:v>
       </x:c>
       <x:c r="H176" s="2">
         <x:v>0</x:v>
@@ -12675,10 +12675,10 @@
       <x:c r="C177" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D177" s="4" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E177" s="4" t="n">
+      <x:c r="D177" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E177" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F177" s="4">
@@ -12734,19 +12734,19 @@
       </x:c>
       <x:c r="D178" s="6" t="n">
         <x:f>SUM(D2:D177)</x:f>
-        <x:v>0</x:v>
+        <x:v>32331.7340073</x:v>
       </x:c>
       <x:c r="E178" s="6" t="n">
         <x:f>SUM(E2:E177)</x:f>
-        <x:v>0</x:v>
+        <x:v>16381.042992609999</x:v>
       </x:c>
       <x:c r="F178" s="6" t="n">
         <x:f>SUM(F2:F177)</x:f>
-        <x:v>0</x:v>
+        <x:v>11700.744994721428</x:v>
       </x:c>
       <x:c r="G178" s="6" t="n">
         <x:f>SUM(G2:G177)</x:f>
-        <x:v>0</x:v>
+        <x:v>28081.78798733143</x:v>
       </x:c>
       <x:c r="T178" s="8" t="n">
         <x:f>SUM(T2:T177)</x:f>

</xml_diff>